<commit_message>
Codigo de automata muy cerca de terminado ademas de que se comienza con la creacion de los registros con la libreria loggin para depuracion auditoria y orden
</commit_message>
<xml_diff>
--- a/Output/040_12e_R11/040_12e_R11_202506.xlsx
+++ b/Output/040_12e_R11/040_12e_R11_202506.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\Usuario\Desktop\TDCBanksMx\Output\040_12e_R11\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\espar\Desktop\Portafolio\TDCBanksMx\Output\040_12e_R11\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{46CBC84B-B812-4FCE-958F-E685F7F5354E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5246711D-5F49-49B5-9B69-2020FDF080C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,12 +20,126 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t>Número de Impagos Consecutivos</t>
   </si>
   <si>
     <t>Actinver</t>
+  </si>
+  <si>
+    <t>Afirme</t>
+  </si>
+  <si>
+    <t>American Express</t>
+  </si>
+  <si>
+    <t>Banamex</t>
+  </si>
+  <si>
+    <t>Banca Mifel</t>
+  </si>
+  <si>
+    <t>Banco Ahorro Famsa</t>
+  </si>
+  <si>
+    <t>Banco Azteca</t>
+  </si>
+  <si>
+    <t>Banco Bineo</t>
+  </si>
+  <si>
+    <t>Banco del Bajío</t>
+  </si>
+  <si>
+    <t>Banco Wal-Mart</t>
+  </si>
+  <si>
+    <t>Bancoppel</t>
+  </si>
+  <si>
+    <t>Banjército</t>
+  </si>
+  <si>
+    <t>Banorte</t>
+  </si>
+  <si>
+    <t>Banorte-Ixe Tarjetas</t>
+  </si>
+  <si>
+    <t>Banregio</t>
+  </si>
+  <si>
+    <t>BBVA México</t>
+  </si>
+  <si>
+    <t>BNP Paribas Personal Finance</t>
+  </si>
+  <si>
+    <t>CIBanco</t>
+  </si>
+  <si>
+    <t>Comercios Afiliados</t>
+  </si>
+  <si>
+    <t>Consubanco</t>
+  </si>
+  <si>
+    <t>Crédito Familiar</t>
+  </si>
+  <si>
+    <t>Dondé Banco</t>
+  </si>
+  <si>
+    <t>Forjadores</t>
+  </si>
+  <si>
+    <t>Globalcard</t>
+  </si>
+  <si>
+    <t>HSBC</t>
+  </si>
+  <si>
+    <t>Interacciones</t>
+  </si>
+  <si>
+    <t>Intercam Banco</t>
+  </si>
+  <si>
+    <t>Invex</t>
+  </si>
+  <si>
+    <t>Invex Consumo</t>
+  </si>
+  <si>
+    <t>Openbank</t>
+  </si>
+  <si>
+    <t>Santander</t>
+  </si>
+  <si>
+    <t>Santander Consumo</t>
+  </si>
+  <si>
+    <t>Santander Inclusión Financiera</t>
+  </si>
+  <si>
+    <t>Scotiabank</t>
+  </si>
+  <si>
+    <t>Servicios Financieros Soriana</t>
+  </si>
+  <si>
+    <t>Sociedad Financiera Inbursa</t>
+  </si>
+  <si>
+    <t>Sofom Inbursa</t>
+  </si>
+  <si>
+    <t>Tarjetas Banamex</t>
+  </si>
+  <si>
+    <t>Ualá</t>
   </si>
   <si>
     <t>Más de 12</t>
@@ -383,23 +497,251 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R18"/>
+  <dimension ref="A1:AO18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:41" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" t="s">
+        <v>11</v>
+      </c>
+      <c r="N1" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" t="s">
+        <v>13</v>
+      </c>
+      <c r="P1" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1" t="s">
+        <v>16</v>
+      </c>
+      <c r="S1" t="s">
+        <v>17</v>
+      </c>
+      <c r="T1" t="s">
+        <v>18</v>
+      </c>
+      <c r="U1" t="s">
+        <v>19</v>
+      </c>
+      <c r="V1" t="s">
+        <v>20</v>
+      </c>
+      <c r="W1" t="s">
+        <v>21</v>
+      </c>
+      <c r="X1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>24</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>34</v>
+      </c>
+      <c r="AK1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AL1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AM1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AN1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AO1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:41" x14ac:dyDescent="0.25">
       <c r="C2">
         <v>202506</v>
       </c>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="D2">
+        <v>202506</v>
+      </c>
+      <c r="E2">
+        <v>202506</v>
+      </c>
+      <c r="F2">
+        <v>202506</v>
+      </c>
+      <c r="G2">
+        <v>202506</v>
+      </c>
+      <c r="H2">
+        <v>202506</v>
+      </c>
+      <c r="I2">
+        <v>202506</v>
+      </c>
+      <c r="J2">
+        <v>202506</v>
+      </c>
+      <c r="K2">
+        <v>202506</v>
+      </c>
+      <c r="L2">
+        <v>202506</v>
+      </c>
+      <c r="M2">
+        <v>202506</v>
+      </c>
+      <c r="N2">
+        <v>202506</v>
+      </c>
+      <c r="O2">
+        <v>202506</v>
+      </c>
+      <c r="P2">
+        <v>202506</v>
+      </c>
+      <c r="Q2">
+        <v>202506</v>
+      </c>
+      <c r="R2">
+        <v>202506</v>
+      </c>
+      <c r="S2">
+        <v>202506</v>
+      </c>
+      <c r="T2">
+        <v>202506</v>
+      </c>
+      <c r="U2">
+        <v>202506</v>
+      </c>
+      <c r="V2">
+        <v>202506</v>
+      </c>
+      <c r="W2">
+        <v>202506</v>
+      </c>
+      <c r="X2">
+        <v>202506</v>
+      </c>
+      <c r="Y2">
+        <v>202506</v>
+      </c>
+      <c r="Z2">
+        <v>202506</v>
+      </c>
+      <c r="AA2">
+        <v>202506</v>
+      </c>
+      <c r="AB2">
+        <v>202506</v>
+      </c>
+      <c r="AC2">
+        <v>202506</v>
+      </c>
+      <c r="AD2">
+        <v>202506</v>
+      </c>
+      <c r="AE2">
+        <v>202506</v>
+      </c>
+      <c r="AF2">
+        <v>202506</v>
+      </c>
+      <c r="AG2">
+        <v>202506</v>
+      </c>
+      <c r="AH2">
+        <v>202506</v>
+      </c>
+      <c r="AI2">
+        <v>202506</v>
+      </c>
+      <c r="AJ2">
+        <v>202506</v>
+      </c>
+      <c r="AK2">
+        <v>202506</v>
+      </c>
+      <c r="AL2">
+        <v>202506</v>
+      </c>
+      <c r="AM2">
+        <v>202506</v>
+      </c>
+      <c r="AN2">
+        <v>202506</v>
+      </c>
+      <c r="AO2">
+        <v>202506</v>
+      </c>
+    </row>
+    <row r="3" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>0</v>
       </c>
@@ -409,8 +751,62 @@
       <c r="C3">
         <v>384</v>
       </c>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="D3">
+        <v>80111</v>
+      </c>
+      <c r="F3">
+        <v>2665</v>
+      </c>
+      <c r="G3">
+        <v>14742</v>
+      </c>
+      <c r="I3">
+        <v>899836</v>
+      </c>
+      <c r="K3">
+        <v>98475</v>
+      </c>
+      <c r="M3">
+        <v>3434706</v>
+      </c>
+      <c r="N3">
+        <v>21188</v>
+      </c>
+      <c r="O3">
+        <v>2712030</v>
+      </c>
+      <c r="Q3">
+        <v>330416</v>
+      </c>
+      <c r="R3">
+        <v>10149067</v>
+      </c>
+      <c r="AA3">
+        <v>2087109</v>
+      </c>
+      <c r="AD3">
+        <v>1113144</v>
+      </c>
+      <c r="AF3">
+        <v>13193</v>
+      </c>
+      <c r="AG3">
+        <v>3783838</v>
+      </c>
+      <c r="AJ3">
+        <v>491047</v>
+      </c>
+      <c r="AM3">
+        <v>1153663</v>
+      </c>
+      <c r="AN3">
+        <v>6721760</v>
+      </c>
+      <c r="AO3">
+        <v>180174</v>
+      </c>
+    </row>
+    <row r="4" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
@@ -420,8 +816,62 @@
       <c r="C4">
         <v>25</v>
       </c>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="D4">
+        <v>3820</v>
+      </c>
+      <c r="F4">
+        <v>316</v>
+      </c>
+      <c r="G4">
+        <v>1268</v>
+      </c>
+      <c r="I4">
+        <v>41311</v>
+      </c>
+      <c r="K4">
+        <v>2706</v>
+      </c>
+      <c r="M4">
+        <v>87450</v>
+      </c>
+      <c r="N4">
+        <v>307</v>
+      </c>
+      <c r="O4">
+        <v>39090</v>
+      </c>
+      <c r="Q4">
+        <v>7678</v>
+      </c>
+      <c r="R4">
+        <v>250823</v>
+      </c>
+      <c r="AA4">
+        <v>69459</v>
+      </c>
+      <c r="AD4">
+        <v>27726</v>
+      </c>
+      <c r="AF4">
+        <v>127</v>
+      </c>
+      <c r="AG4">
+        <v>70952</v>
+      </c>
+      <c r="AJ4">
+        <v>9381</v>
+      </c>
+      <c r="AM4">
+        <v>12799</v>
+      </c>
+      <c r="AN4">
+        <v>153878</v>
+      </c>
+      <c r="AO4">
+        <v>8425</v>
+      </c>
+    </row>
+    <row r="5" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2</v>
       </c>
@@ -431,8 +881,62 @@
       <c r="C5">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="D5">
+        <v>1748</v>
+      </c>
+      <c r="F5">
+        <v>282</v>
+      </c>
+      <c r="G5">
+        <v>203</v>
+      </c>
+      <c r="I5">
+        <v>10048</v>
+      </c>
+      <c r="K5">
+        <v>1153</v>
+      </c>
+      <c r="M5">
+        <v>37592</v>
+      </c>
+      <c r="N5">
+        <v>102</v>
+      </c>
+      <c r="O5">
+        <v>30002</v>
+      </c>
+      <c r="Q5">
+        <v>3149</v>
+      </c>
+      <c r="R5">
+        <v>115812</v>
+      </c>
+      <c r="AA5">
+        <v>30148</v>
+      </c>
+      <c r="AD5">
+        <v>20687</v>
+      </c>
+      <c r="AF5">
+        <v>21</v>
+      </c>
+      <c r="AG5">
+        <v>24130</v>
+      </c>
+      <c r="AJ5">
+        <v>4095</v>
+      </c>
+      <c r="AM5">
+        <v>11967</v>
+      </c>
+      <c r="AN5">
+        <v>57893</v>
+      </c>
+      <c r="AO5">
+        <v>6175</v>
+      </c>
+    </row>
+    <row r="6" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>3</v>
       </c>
@@ -442,8 +946,65 @@
       <c r="C6">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="D6">
+        <v>910</v>
+      </c>
+      <c r="F6">
+        <v>26</v>
+      </c>
+      <c r="G6">
+        <v>176</v>
+      </c>
+      <c r="I6">
+        <v>7336</v>
+      </c>
+      <c r="K6">
+        <v>650</v>
+      </c>
+      <c r="M6">
+        <v>25828</v>
+      </c>
+      <c r="N6">
+        <v>103</v>
+      </c>
+      <c r="O6">
+        <v>19989</v>
+      </c>
+      <c r="Q6">
+        <v>1988</v>
+      </c>
+      <c r="R6">
+        <v>78724</v>
+      </c>
+      <c r="AA6">
+        <v>17706</v>
+      </c>
+      <c r="AD6">
+        <v>12041</v>
+      </c>
+      <c r="AF6">
+        <v>3</v>
+      </c>
+      <c r="AG6">
+        <v>18390</v>
+      </c>
+      <c r="AI6">
+        <v>1</v>
+      </c>
+      <c r="AJ6">
+        <v>2686</v>
+      </c>
+      <c r="AM6">
+        <v>4667</v>
+      </c>
+      <c r="AN6">
+        <v>38891</v>
+      </c>
+      <c r="AO6">
+        <v>5084</v>
+      </c>
+    </row>
+    <row r="7" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>4</v>
       </c>
@@ -453,8 +1014,56 @@
       <c r="C7">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="D7">
+        <v>791</v>
+      </c>
+      <c r="F7">
+        <v>10</v>
+      </c>
+      <c r="I7">
+        <v>5968</v>
+      </c>
+      <c r="K7">
+        <v>440</v>
+      </c>
+      <c r="M7">
+        <v>22870</v>
+      </c>
+      <c r="N7">
+        <v>88</v>
+      </c>
+      <c r="O7">
+        <v>20756</v>
+      </c>
+      <c r="Q7">
+        <v>1789</v>
+      </c>
+      <c r="R7">
+        <v>89813</v>
+      </c>
+      <c r="AA7">
+        <v>15758</v>
+      </c>
+      <c r="AD7">
+        <v>11041</v>
+      </c>
+      <c r="AG7">
+        <v>21250</v>
+      </c>
+      <c r="AJ7">
+        <v>2637</v>
+      </c>
+      <c r="AM7">
+        <v>5962</v>
+      </c>
+      <c r="AN7">
+        <v>38885</v>
+      </c>
+      <c r="AO7">
+        <v>3154</v>
+      </c>
+    </row>
+    <row r="8" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>5</v>
       </c>
@@ -464,8 +1073,56 @@
       <c r="C8">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="D8">
+        <v>820</v>
+      </c>
+      <c r="F8">
+        <v>9</v>
+      </c>
+      <c r="I8">
+        <v>5830</v>
+      </c>
+      <c r="K8">
+        <v>439</v>
+      </c>
+      <c r="M8">
+        <v>21477</v>
+      </c>
+      <c r="N8">
+        <v>103</v>
+      </c>
+      <c r="O8">
+        <v>18880</v>
+      </c>
+      <c r="Q8">
+        <v>1639</v>
+      </c>
+      <c r="R8">
+        <v>27537</v>
+      </c>
+      <c r="AA8">
+        <v>13153</v>
+      </c>
+      <c r="AD8">
+        <v>10636</v>
+      </c>
+      <c r="AG8">
+        <v>19291</v>
+      </c>
+      <c r="AJ8">
+        <v>2312</v>
+      </c>
+      <c r="AM8">
+        <v>7</v>
+      </c>
+      <c r="AN8">
+        <v>35166</v>
+      </c>
+      <c r="AO8">
+        <v>2829</v>
+      </c>
+    </row>
+    <row r="9" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>6</v>
       </c>
@@ -475,8 +1132,53 @@
       <c r="C9">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="D9">
+        <v>248</v>
+      </c>
+      <c r="F9">
+        <v>10</v>
+      </c>
+      <c r="I9">
+        <v>5721</v>
+      </c>
+      <c r="K9">
+        <v>414</v>
+      </c>
+      <c r="M9">
+        <v>17443</v>
+      </c>
+      <c r="N9">
+        <v>71</v>
+      </c>
+      <c r="O9">
+        <v>3</v>
+      </c>
+      <c r="Q9">
+        <v>1370</v>
+      </c>
+      <c r="R9">
+        <v>14416</v>
+      </c>
+      <c r="AA9">
+        <v>11184</v>
+      </c>
+      <c r="AD9">
+        <v>2127</v>
+      </c>
+      <c r="AG9">
+        <v>6403</v>
+      </c>
+      <c r="AJ9">
+        <v>1811</v>
+      </c>
+      <c r="AN9">
+        <v>30369</v>
+      </c>
+      <c r="AO9">
+        <v>2466</v>
+      </c>
+    </row>
+    <row r="10" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>7</v>
       </c>
@@ -486,8 +1188,53 @@
       <c r="C10">
         <v>3</v>
       </c>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="D10">
+        <v>152</v>
+      </c>
+      <c r="F10">
+        <v>10</v>
+      </c>
+      <c r="I10">
+        <v>5551</v>
+      </c>
+      <c r="K10">
+        <v>110</v>
+      </c>
+      <c r="M10">
+        <v>15932</v>
+      </c>
+      <c r="N10">
+        <v>44</v>
+      </c>
+      <c r="O10">
+        <v>5</v>
+      </c>
+      <c r="Q10">
+        <v>653</v>
+      </c>
+      <c r="R10">
+        <v>7699</v>
+      </c>
+      <c r="AA10">
+        <v>3651</v>
+      </c>
+      <c r="AD10">
+        <v>746</v>
+      </c>
+      <c r="AG10">
+        <v>4165</v>
+      </c>
+      <c r="AJ10">
+        <v>690</v>
+      </c>
+      <c r="AN10">
+        <v>4180</v>
+      </c>
+      <c r="AO10">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="11" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>8</v>
       </c>
@@ -497,9 +1244,53 @@
       <c r="C11">
         <v>2</v>
       </c>
-      <c r="R11" s="1"/>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="D11">
+        <v>114</v>
+      </c>
+      <c r="F11">
+        <v>13</v>
+      </c>
+      <c r="I11">
+        <v>3220</v>
+      </c>
+      <c r="K11">
+        <v>54</v>
+      </c>
+      <c r="M11">
+        <v>7858</v>
+      </c>
+      <c r="N11">
+        <v>55</v>
+      </c>
+      <c r="O11">
+        <v>4</v>
+      </c>
+      <c r="Q11">
+        <v>601</v>
+      </c>
+      <c r="R11" s="1">
+        <v>4519</v>
+      </c>
+      <c r="AA11">
+        <v>1507</v>
+      </c>
+      <c r="AD11">
+        <v>534</v>
+      </c>
+      <c r="AG11">
+        <v>1920</v>
+      </c>
+      <c r="AJ11">
+        <v>386</v>
+      </c>
+      <c r="AN11">
+        <v>2114</v>
+      </c>
+      <c r="AO11">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="12" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>9</v>
       </c>
@@ -509,56 +1300,287 @@
       <c r="C12">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="D12">
+        <v>79</v>
+      </c>
+      <c r="F12">
+        <v>12</v>
+      </c>
+      <c r="K12">
+        <v>44</v>
+      </c>
+      <c r="M12">
+        <v>6822</v>
+      </c>
+      <c r="N12">
+        <v>31</v>
+      </c>
+      <c r="O12">
+        <v>199</v>
+      </c>
+      <c r="Q12">
+        <v>272</v>
+      </c>
+      <c r="R12">
+        <v>3740</v>
+      </c>
+      <c r="AA12">
+        <v>748</v>
+      </c>
+      <c r="AD12">
+        <v>231</v>
+      </c>
+      <c r="AG12">
+        <v>2052</v>
+      </c>
+      <c r="AJ12">
+        <v>270</v>
+      </c>
+      <c r="AN12">
+        <v>1045</v>
+      </c>
+      <c r="AO12">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="13" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>10</v>
       </c>
       <c r="B13">
         <v>10</v>
       </c>
-    </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="D13">
+        <v>56</v>
+      </c>
+      <c r="F13">
+        <v>2</v>
+      </c>
+      <c r="I13">
+        <v>1</v>
+      </c>
+      <c r="K13">
+        <v>32</v>
+      </c>
+      <c r="M13">
+        <v>9617</v>
+      </c>
+      <c r="N13">
+        <v>48</v>
+      </c>
+      <c r="Q13">
+        <v>175</v>
+      </c>
+      <c r="R13">
+        <v>2705</v>
+      </c>
+      <c r="AA13">
+        <v>445</v>
+      </c>
+      <c r="AD13">
+        <v>133</v>
+      </c>
+      <c r="AG13">
+        <v>1620</v>
+      </c>
+      <c r="AJ13">
+        <v>231</v>
+      </c>
+      <c r="AN13">
+        <v>716</v>
+      </c>
+      <c r="AO13">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>11</v>
       </c>
       <c r="B14">
         <v>11</v>
       </c>
-    </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="D14">
+        <v>36</v>
+      </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="K14">
+        <v>31</v>
+      </c>
+      <c r="M14">
+        <v>6928</v>
+      </c>
+      <c r="N14">
+        <v>33</v>
+      </c>
+      <c r="Q14">
+        <v>135</v>
+      </c>
+      <c r="R14">
+        <v>2585</v>
+      </c>
+      <c r="AA14">
+        <v>228</v>
+      </c>
+      <c r="AD14">
+        <v>65</v>
+      </c>
+      <c r="AG14">
+        <v>1598</v>
+      </c>
+      <c r="AJ14">
+        <v>149</v>
+      </c>
+      <c r="AN14">
+        <v>400</v>
+      </c>
+      <c r="AO14">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>12</v>
       </c>
       <c r="B15">
         <v>12</v>
       </c>
-    </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="D15">
+        <v>113</v>
+      </c>
+      <c r="F15">
+        <v>2</v>
+      </c>
+      <c r="K15">
+        <v>49</v>
+      </c>
+      <c r="M15">
+        <v>6036</v>
+      </c>
+      <c r="N15">
+        <v>29</v>
+      </c>
+      <c r="Q15">
+        <v>748</v>
+      </c>
+      <c r="R15">
+        <v>16779</v>
+      </c>
+      <c r="AA15">
+        <v>5730</v>
+      </c>
+      <c r="AD15">
+        <v>108</v>
+      </c>
+      <c r="AG15">
+        <v>28655</v>
+      </c>
+      <c r="AJ15">
+        <v>944</v>
+      </c>
+      <c r="AN15">
+        <v>757</v>
+      </c>
+      <c r="AO15">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>13</v>
       </c>
       <c r="B16" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="C16">
         <v>7</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="K16">
+        <v>2</v>
+      </c>
+      <c r="M16">
+        <v>32839</v>
+      </c>
+      <c r="N16">
+        <v>298</v>
+      </c>
+      <c r="AG16">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>999</v>
       </c>
       <c r="B17" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="18" spans="1:41" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
-        <v>4</v>
+        <v>42</v>
       </c>
       <c r="C18">
         <v>430</v>
+      </c>
+      <c r="D18">
+        <v>88998</v>
+      </c>
+      <c r="F18">
+        <v>3358</v>
+      </c>
+      <c r="G18">
+        <v>16389</v>
+      </c>
+      <c r="I18">
+        <v>984822</v>
+      </c>
+      <c r="K18">
+        <v>104599</v>
+      </c>
+      <c r="M18">
+        <v>3733398</v>
+      </c>
+      <c r="N18">
+        <v>22500</v>
+      </c>
+      <c r="O18">
+        <v>2840958</v>
+      </c>
+      <c r="Q18">
+        <v>350613</v>
+      </c>
+      <c r="R18">
+        <v>10764219</v>
+      </c>
+      <c r="AA18">
+        <v>2256826</v>
+      </c>
+      <c r="AD18">
+        <v>1199219</v>
+      </c>
+      <c r="AF18">
+        <v>13344</v>
+      </c>
+      <c r="AG18">
+        <v>3984270</v>
+      </c>
+      <c r="AI18">
+        <v>1</v>
+      </c>
+      <c r="AJ18">
+        <v>516639</v>
+      </c>
+      <c r="AM18">
+        <v>1189065</v>
+      </c>
+      <c r="AN18">
+        <v>7086054</v>
+      </c>
+      <c r="AO18">
+        <v>208857</v>
       </c>
     </row>
   </sheetData>

</xml_diff>